<commit_message>
logs: update NSE signals 2026-09-14
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X88"/>
+  <dimension ref="A1:X89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2721,9 +2721,16 @@
         </is>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-09-14  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="68">
+  <mergeCells count="69">
     <mergeCell ref="A79:X79"/>
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A87:X87"/>
@@ -2737,6 +2744,7 @@
     <mergeCell ref="A46:X46"/>
     <mergeCell ref="A84:X84"/>
     <mergeCell ref="A66:X66"/>
+    <mergeCell ref="A89:X89"/>
     <mergeCell ref="A74:X74"/>
     <mergeCell ref="A80:X80"/>
     <mergeCell ref="A56:X56"/>
@@ -16878,7 +16886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I71"/>
+  <dimension ref="A1:I72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19040,6 +19048,36 @@
         <v>0</v>
       </c>
       <c r="H71" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="18" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B72" s="19" t="n">
+        <v>7</v>
+      </c>
+      <c r="C72" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D72" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E72" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F72" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G72" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H72" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-09-15
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X89"/>
+  <dimension ref="A1:X90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2728,9 +2728,16 @@
         </is>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-09-15  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="69">
+  <mergeCells count="70">
     <mergeCell ref="A79:X79"/>
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A87:X87"/>
@@ -2739,11 +2746,12 @@
     <mergeCell ref="A54:X54"/>
     <mergeCell ref="A25:X25"/>
     <mergeCell ref="A41:X41"/>
+    <mergeCell ref="A90:X90"/>
     <mergeCell ref="A75:X75"/>
     <mergeCell ref="A37:X37"/>
     <mergeCell ref="A46:X46"/>
+    <mergeCell ref="A66:X66"/>
     <mergeCell ref="A84:X84"/>
-    <mergeCell ref="A66:X66"/>
     <mergeCell ref="A89:X89"/>
     <mergeCell ref="A74:X74"/>
     <mergeCell ref="A80:X80"/>
@@ -16886,7 +16894,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I72"/>
+  <dimension ref="A1:I73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19078,6 +19086,36 @@
         <v>0</v>
       </c>
       <c r="H72" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="18" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B73" s="19" t="n">
+        <v>11</v>
+      </c>
+      <c r="C73" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D73" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E73" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F73" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G73" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-09-16
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X90"/>
+  <dimension ref="A1:X91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2735,9 +2735,16 @@
         </is>
       </c>
     </row>
+    <row r="91">
+      <c r="A91" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-09-16  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="70">
+  <mergeCells count="71">
     <mergeCell ref="A79:X79"/>
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A87:X87"/>
@@ -2772,6 +2779,7 @@
     <mergeCell ref="A32:X32"/>
     <mergeCell ref="A22:X22"/>
     <mergeCell ref="A53:X53"/>
+    <mergeCell ref="A91:X91"/>
     <mergeCell ref="A29:X29"/>
     <mergeCell ref="A35:X35"/>
     <mergeCell ref="A62:X62"/>
@@ -16894,7 +16902,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I73"/>
+  <dimension ref="A1:I74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19116,6 +19124,36 @@
         <v>0</v>
       </c>
       <c r="H73" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="18" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B74" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="C74" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D74" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E74" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F74" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G74" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H74" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-09-17
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X91"/>
+  <dimension ref="A1:X92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2742,9 +2742,16 @@
         </is>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-09-17  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="71">
+  <mergeCells count="72">
     <mergeCell ref="A79:X79"/>
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A87:X87"/>
@@ -2796,6 +2803,7 @@
     <mergeCell ref="A58:X58"/>
     <mergeCell ref="A40:X40"/>
     <mergeCell ref="A67:X67"/>
+    <mergeCell ref="A92:X92"/>
     <mergeCell ref="A30:X30"/>
     <mergeCell ref="A39:X39"/>
     <mergeCell ref="A34:X34"/>
@@ -16902,7 +16910,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I74"/>
+  <dimension ref="A1:I75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19154,6 +19162,36 @@
         <v>0</v>
       </c>
       <c r="H74" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="18" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B75" s="19" t="n">
+        <v>11</v>
+      </c>
+      <c r="C75" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D75" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E75" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F75" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G75" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H75" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-09-18
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X92"/>
+  <dimension ref="A1:X93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2749,9 +2749,16 @@
         </is>
       </c>
     </row>
+    <row r="93">
+      <c r="A93" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-09-18  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="72">
+  <mergeCells count="73">
     <mergeCell ref="A79:X79"/>
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A87:X87"/>
@@ -2798,6 +2805,7 @@
     <mergeCell ref="A28:X28"/>
     <mergeCell ref="A68:X68"/>
     <mergeCell ref="A63:X63"/>
+    <mergeCell ref="A93:X93"/>
     <mergeCell ref="A31:X31"/>
     <mergeCell ref="A44:X44"/>
     <mergeCell ref="A58:X58"/>
@@ -16910,7 +16918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I75"/>
+  <dimension ref="A1:I76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19192,6 +19200,36 @@
         <v>0</v>
       </c>
       <c r="H75" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="18" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B76" s="19" t="n">
+        <v>16</v>
+      </c>
+      <c r="C76" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D76" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E76" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F76" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G76" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H76" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-09-21
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X93"/>
+  <dimension ref="A1:X94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2756,9 +2756,16 @@
         </is>
       </c>
     </row>
+    <row r="94">
+      <c r="A94" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-09-21  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="73">
+  <mergeCells count="74">
     <mergeCell ref="A79:X79"/>
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A87:X87"/>
@@ -2827,6 +2834,7 @@
     <mergeCell ref="A49:X49"/>
     <mergeCell ref="A51:X51"/>
     <mergeCell ref="A45:X45"/>
+    <mergeCell ref="A94:X94"/>
     <mergeCell ref="A21:V21"/>
     <mergeCell ref="A36:X36"/>
     <mergeCell ref="A61:X61"/>
@@ -16918,7 +16926,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I76"/>
+  <dimension ref="A1:I77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19230,6 +19238,36 @@
         <v>0</v>
       </c>
       <c r="H76" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="18" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B77" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="C77" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D77" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E77" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F77" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G77" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H77" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-09-22
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X94"/>
+  <dimension ref="A1:X95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2763,9 +2763,16 @@
         </is>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-09-22  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="74">
+  <mergeCells count="75">
     <mergeCell ref="A79:X79"/>
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A87:X87"/>
@@ -2789,6 +2796,7 @@
     <mergeCell ref="A50:X50"/>
     <mergeCell ref="A26:X26"/>
     <mergeCell ref="A57:X57"/>
+    <mergeCell ref="A95:X95"/>
     <mergeCell ref="A86:X86"/>
     <mergeCell ref="A42:X42"/>
     <mergeCell ref="A76:X76"/>
@@ -16926,7 +16934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I77"/>
+  <dimension ref="A1:I78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19268,6 +19276,36 @@
         <v>0</v>
       </c>
       <c r="H77" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="18" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B78" s="19" t="n">
+        <v>13</v>
+      </c>
+      <c r="C78" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D78" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E78" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F78" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G78" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H78" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-09-23
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X95"/>
+  <dimension ref="A1:X96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2770,9 +2770,16 @@
         </is>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-09-23  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="75">
+  <mergeCells count="76">
     <mergeCell ref="A79:X79"/>
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A87:X87"/>
@@ -2817,6 +2824,7 @@
     <mergeCell ref="A81:X81"/>
     <mergeCell ref="A72:X72"/>
     <mergeCell ref="A52:X52"/>
+    <mergeCell ref="A96:X96"/>
     <mergeCell ref="A28:X28"/>
     <mergeCell ref="A68:X68"/>
     <mergeCell ref="A63:X63"/>
@@ -16934,7 +16942,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I78"/>
+  <dimension ref="A1:I79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19306,6 +19314,36 @@
         <v>0</v>
       </c>
       <c r="H78" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="18" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B79" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="C79" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D79" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E79" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F79" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G79" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H79" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-09-24
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X96"/>
+  <dimension ref="A1:X97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2777,85 +2777,93 @@
         </is>
       </c>
     </row>
+    <row r="97">
+      <c r="A97" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-09-24  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="76">
-    <mergeCell ref="A79:X79"/>
+  <mergeCells count="77">
     <mergeCell ref="A69:X69"/>
-    <mergeCell ref="A87:X87"/>
-    <mergeCell ref="A65:X65"/>
     <mergeCell ref="A78:X78"/>
-    <mergeCell ref="A54:X54"/>
-    <mergeCell ref="A25:X25"/>
-    <mergeCell ref="A41:X41"/>
-    <mergeCell ref="A90:X90"/>
     <mergeCell ref="A75:X75"/>
-    <mergeCell ref="A37:X37"/>
-    <mergeCell ref="A46:X46"/>
-    <mergeCell ref="A66:X66"/>
-    <mergeCell ref="A84:X84"/>
-    <mergeCell ref="A89:X89"/>
-    <mergeCell ref="A74:X74"/>
     <mergeCell ref="A80:X80"/>
-    <mergeCell ref="A56:X56"/>
-    <mergeCell ref="A27:X27"/>
     <mergeCell ref="A55:X55"/>
-    <mergeCell ref="A50:X50"/>
-    <mergeCell ref="A26:X26"/>
-    <mergeCell ref="A57:X57"/>
     <mergeCell ref="A95:X95"/>
-    <mergeCell ref="A86:X86"/>
-    <mergeCell ref="A42:X42"/>
-    <mergeCell ref="A76:X76"/>
-    <mergeCell ref="A33:X33"/>
-    <mergeCell ref="A71:X71"/>
-    <mergeCell ref="A47:X47"/>
-    <mergeCell ref="A85:X85"/>
-    <mergeCell ref="A23:X23"/>
     <mergeCell ref="A32:X32"/>
-    <mergeCell ref="A22:X22"/>
-    <mergeCell ref="A53:X53"/>
-    <mergeCell ref="A91:X91"/>
+    <mergeCell ref="A97:X97"/>
     <mergeCell ref="A29:X29"/>
-    <mergeCell ref="A35:X35"/>
-    <mergeCell ref="A62:X62"/>
-    <mergeCell ref="A43:X43"/>
+    <mergeCell ref="A81:X81"/>
     <mergeCell ref="A38:X38"/>
-    <mergeCell ref="A81:X81"/>
-    <mergeCell ref="A72:X72"/>
-    <mergeCell ref="A52:X52"/>
     <mergeCell ref="A96:X96"/>
-    <mergeCell ref="A28:X28"/>
-    <mergeCell ref="A68:X68"/>
-    <mergeCell ref="A63:X63"/>
-    <mergeCell ref="A93:X93"/>
     <mergeCell ref="A31:X31"/>
-    <mergeCell ref="A44:X44"/>
     <mergeCell ref="A58:X58"/>
     <mergeCell ref="A40:X40"/>
     <mergeCell ref="A67:X67"/>
-    <mergeCell ref="A92:X92"/>
-    <mergeCell ref="A30:X30"/>
-    <mergeCell ref="A39:X39"/>
-    <mergeCell ref="A34:X34"/>
-    <mergeCell ref="A77:X77"/>
-    <mergeCell ref="A59:X59"/>
-    <mergeCell ref="A48:X48"/>
-    <mergeCell ref="A83:X83"/>
     <mergeCell ref="A24:X24"/>
     <mergeCell ref="A73:X73"/>
-    <mergeCell ref="A64:X64"/>
     <mergeCell ref="A82:X82"/>
     <mergeCell ref="A60:X60"/>
-    <mergeCell ref="A49:X49"/>
+    <mergeCell ref="A25:X25"/>
+    <mergeCell ref="A84:X84"/>
+    <mergeCell ref="A66:X66"/>
+    <mergeCell ref="A50:X50"/>
+    <mergeCell ref="A86:X86"/>
+    <mergeCell ref="A42:X42"/>
+    <mergeCell ref="A47:X47"/>
+    <mergeCell ref="A22:X22"/>
+    <mergeCell ref="A72:X72"/>
+    <mergeCell ref="A28:X28"/>
+    <mergeCell ref="A44:X44"/>
+    <mergeCell ref="A30:X30"/>
+    <mergeCell ref="A59:X59"/>
+    <mergeCell ref="A64:X64"/>
     <mergeCell ref="A51:X51"/>
+    <mergeCell ref="A61:X61"/>
+    <mergeCell ref="A88:X88"/>
+    <mergeCell ref="A70:X70"/>
+    <mergeCell ref="A54:X54"/>
+    <mergeCell ref="A41:X41"/>
+    <mergeCell ref="A90:X90"/>
+    <mergeCell ref="A74:X74"/>
+    <mergeCell ref="A56:X56"/>
+    <mergeCell ref="A27:X27"/>
+    <mergeCell ref="A76:X76"/>
+    <mergeCell ref="A33:X33"/>
+    <mergeCell ref="A85:X85"/>
+    <mergeCell ref="A53:X53"/>
+    <mergeCell ref="A35:X35"/>
+    <mergeCell ref="A62:X62"/>
+    <mergeCell ref="A68:X68"/>
+    <mergeCell ref="A92:X92"/>
+    <mergeCell ref="A39:X39"/>
+    <mergeCell ref="A48:X48"/>
     <mergeCell ref="A45:X45"/>
     <mergeCell ref="A94:X94"/>
     <mergeCell ref="A21:V21"/>
+    <mergeCell ref="A79:X79"/>
+    <mergeCell ref="A87:X87"/>
+    <mergeCell ref="A65:X65"/>
+    <mergeCell ref="A37:X37"/>
+    <mergeCell ref="A46:X46"/>
+    <mergeCell ref="A89:X89"/>
+    <mergeCell ref="A26:X26"/>
+    <mergeCell ref="A57:X57"/>
+    <mergeCell ref="A71:X71"/>
+    <mergeCell ref="A23:X23"/>
+    <mergeCell ref="A91:X91"/>
+    <mergeCell ref="A43:X43"/>
+    <mergeCell ref="A52:X52"/>
+    <mergeCell ref="A63:X63"/>
+    <mergeCell ref="A93:X93"/>
+    <mergeCell ref="A77:X77"/>
+    <mergeCell ref="A34:X34"/>
+    <mergeCell ref="A83:X83"/>
+    <mergeCell ref="A49:X49"/>
     <mergeCell ref="A36:X36"/>
-    <mergeCell ref="A61:X61"/>
-    <mergeCell ref="A88:X88"/>
-    <mergeCell ref="A70:X70"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16942,7 +16950,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I79"/>
+  <dimension ref="A1:I80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19344,6 +19352,36 @@
         <v>0</v>
       </c>
       <c r="H79" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="18" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B80" s="19" t="n">
+        <v>13</v>
+      </c>
+      <c r="C80" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D80" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E80" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F80" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G80" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H80" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-09-25
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X97"/>
+  <dimension ref="A1:X98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2784,9 +2784,16 @@
         </is>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-09-25  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="77">
+  <mergeCells count="78">
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A78:X78"/>
     <mergeCell ref="A75:X75"/>
@@ -2821,6 +2828,7 @@
     <mergeCell ref="A30:X30"/>
     <mergeCell ref="A59:X59"/>
     <mergeCell ref="A64:X64"/>
+    <mergeCell ref="A98:X98"/>
     <mergeCell ref="A51:X51"/>
     <mergeCell ref="A61:X61"/>
     <mergeCell ref="A88:X88"/>
@@ -16950,7 +16958,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I80"/>
+  <dimension ref="A1:I81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19382,6 +19390,36 @@
         <v>0</v>
       </c>
       <c r="H80" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="18" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B81" s="19" t="n">
+        <v>9</v>
+      </c>
+      <c r="C81" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D81" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E81" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F81" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G81" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H81" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-10-14
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X98"/>
+  <dimension ref="A1:X99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2791,9 +2791,16 @@
         </is>
       </c>
     </row>
+    <row r="99">
+      <c r="A99" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-10-14  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="78">
+  <mergeCells count="79">
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A78:X78"/>
     <mergeCell ref="A75:X75"/>
@@ -2836,6 +2843,7 @@
     <mergeCell ref="A54:X54"/>
     <mergeCell ref="A41:X41"/>
     <mergeCell ref="A90:X90"/>
+    <mergeCell ref="A99:X99"/>
     <mergeCell ref="A74:X74"/>
     <mergeCell ref="A56:X56"/>
     <mergeCell ref="A27:X27"/>
@@ -16958,7 +16966,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I81"/>
+  <dimension ref="A1:I82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19420,6 +19428,36 @@
         <v>0</v>
       </c>
       <c r="H81" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B82" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="C82" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D82" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E82" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F82" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G82" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H82" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-10-15
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X99"/>
+  <dimension ref="A1:X100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2798,9 +2798,16 @@
         </is>
       </c>
     </row>
+    <row r="100">
+      <c r="A100" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-10-15  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="79">
+  <mergeCells count="80">
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A78:X78"/>
     <mergeCell ref="A75:X75"/>
@@ -2871,6 +2878,7 @@
     <mergeCell ref="A71:X71"/>
     <mergeCell ref="A23:X23"/>
     <mergeCell ref="A91:X91"/>
+    <mergeCell ref="A100:X100"/>
     <mergeCell ref="A43:X43"/>
     <mergeCell ref="A52:X52"/>
     <mergeCell ref="A63:X63"/>
@@ -16966,7 +16974,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I82"/>
+  <dimension ref="A1:I83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19458,6 +19466,36 @@
         <v>0</v>
       </c>
       <c r="H82" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B83" s="19" t="n">
+        <v>15</v>
+      </c>
+      <c r="C83" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D83" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E83" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F83" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G83" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H83" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-10-16
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X100"/>
+  <dimension ref="A1:X101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2805,9 +2805,16 @@
         </is>
       </c>
     </row>
+    <row r="101">
+      <c r="A101" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-10-16  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="80">
+  <mergeCells count="81">
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A78:X78"/>
     <mergeCell ref="A75:X75"/>
@@ -2854,6 +2861,7 @@
     <mergeCell ref="A74:X74"/>
     <mergeCell ref="A56:X56"/>
     <mergeCell ref="A27:X27"/>
+    <mergeCell ref="A101:X101"/>
     <mergeCell ref="A76:X76"/>
     <mergeCell ref="A33:X33"/>
     <mergeCell ref="A85:X85"/>
@@ -16974,7 +16982,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I83"/>
+  <dimension ref="A1:I84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19496,6 +19504,36 @@
         <v>0</v>
       </c>
       <c r="H83" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B84" s="19" t="n">
+        <v>16</v>
+      </c>
+      <c r="C84" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D84" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E84" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F84" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-10-19
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X101"/>
+  <dimension ref="A1:X102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2812,9 +2812,16 @@
         </is>
       </c>
     </row>
+    <row r="102">
+      <c r="A102" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-10-19  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="81">
+  <mergeCells count="82">
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A78:X78"/>
     <mergeCell ref="A75:X75"/>
@@ -2869,6 +2876,7 @@
     <mergeCell ref="A35:X35"/>
     <mergeCell ref="A62:X62"/>
     <mergeCell ref="A68:X68"/>
+    <mergeCell ref="A102:X102"/>
     <mergeCell ref="A92:X92"/>
     <mergeCell ref="A39:X39"/>
     <mergeCell ref="A48:X48"/>
@@ -16982,7 +16990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I84"/>
+  <dimension ref="A1:I85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19534,6 +19542,36 @@
         <v>0</v>
       </c>
       <c r="H84" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B85" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="C85" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D85" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E85" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F85" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G85" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H85" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-10-20
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X102"/>
+  <dimension ref="A1:X103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2819,9 +2819,16 @@
         </is>
       </c>
     </row>
+    <row r="103">
+      <c r="A103" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-10-20  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="82">
+  <mergeCells count="83">
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A78:X78"/>
     <mergeCell ref="A75:X75"/>
@@ -2883,6 +2890,7 @@
     <mergeCell ref="A45:X45"/>
     <mergeCell ref="A94:X94"/>
     <mergeCell ref="A21:V21"/>
+    <mergeCell ref="A103:X103"/>
     <mergeCell ref="A79:X79"/>
     <mergeCell ref="A87:X87"/>
     <mergeCell ref="A65:X65"/>
@@ -16990,7 +16998,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I85"/>
+  <dimension ref="A1:I86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19572,6 +19580,36 @@
         <v>0</v>
       </c>
       <c r="H85" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B86" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="C86" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D86" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E86" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F86" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G86" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-10-21
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X103"/>
+  <dimension ref="A1:X104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2826,15 +2826,23 @@
         </is>
       </c>
     </row>
+    <row r="104">
+      <c r="A104" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-10-21  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="83">
+  <mergeCells count="84">
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A78:X78"/>
     <mergeCell ref="A75:X75"/>
     <mergeCell ref="A80:X80"/>
     <mergeCell ref="A55:X55"/>
     <mergeCell ref="A95:X95"/>
+    <mergeCell ref="A104:X104"/>
     <mergeCell ref="A32:X32"/>
     <mergeCell ref="A97:X97"/>
     <mergeCell ref="A29:X29"/>
@@ -16998,7 +17006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I86"/>
+  <dimension ref="A1:I87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19610,6 +19618,36 @@
         <v>0</v>
       </c>
       <c r="H86" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B87" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="C87" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D87" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E87" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F87" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G87" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H87" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-10-22
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X104"/>
+  <dimension ref="A1:X105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2833,9 +2833,16 @@
         </is>
       </c>
     </row>
+    <row r="105">
+      <c r="A105" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-10-22  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="84">
+  <mergeCells count="85">
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A78:X78"/>
     <mergeCell ref="A75:X75"/>
@@ -2905,6 +2912,7 @@
     <mergeCell ref="A37:X37"/>
     <mergeCell ref="A46:X46"/>
     <mergeCell ref="A89:X89"/>
+    <mergeCell ref="A105:X105"/>
     <mergeCell ref="A26:X26"/>
     <mergeCell ref="A57:X57"/>
     <mergeCell ref="A71:X71"/>
@@ -17006,7 +17014,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I87"/>
+  <dimension ref="A1:I88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19648,6 +19656,36 @@
         <v>0</v>
       </c>
       <c r="H87" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B88" s="19" t="n">
+        <v>11</v>
+      </c>
+      <c r="C88" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D88" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E88" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F88" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G88" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H88" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-10-23
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X105"/>
+  <dimension ref="A1:X106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2840,9 +2840,16 @@
         </is>
       </c>
     </row>
+    <row r="106">
+      <c r="A106" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-10-23  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="85">
+  <mergeCells count="86">
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A78:X78"/>
     <mergeCell ref="A75:X75"/>
@@ -2852,6 +2859,7 @@
     <mergeCell ref="A104:X104"/>
     <mergeCell ref="A32:X32"/>
     <mergeCell ref="A97:X97"/>
+    <mergeCell ref="A106:X106"/>
     <mergeCell ref="A29:X29"/>
     <mergeCell ref="A81:X81"/>
     <mergeCell ref="A38:X38"/>
@@ -17014,7 +17022,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I88"/>
+  <dimension ref="A1:I89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19686,6 +19694,36 @@
         <v>0</v>
       </c>
       <c r="H88" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B89" s="19" t="n">
+        <v>12</v>
+      </c>
+      <c r="C89" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D89" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E89" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F89" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G89" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H89" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-10-26
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X106"/>
+  <dimension ref="A1:X107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2847,9 +2847,16 @@
         </is>
       </c>
     </row>
+    <row r="107">
+      <c r="A107" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-10-26  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="86">
+  <mergeCells count="87">
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A78:X78"/>
     <mergeCell ref="A75:X75"/>
@@ -2888,6 +2895,7 @@
     <mergeCell ref="A64:X64"/>
     <mergeCell ref="A98:X98"/>
     <mergeCell ref="A51:X51"/>
+    <mergeCell ref="A107:X107"/>
     <mergeCell ref="A61:X61"/>
     <mergeCell ref="A88:X88"/>
     <mergeCell ref="A70:X70"/>
@@ -17022,7 +17030,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I89"/>
+  <dimension ref="A1:I90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19724,6 +19732,36 @@
         <v>0</v>
       </c>
       <c r="H89" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B90" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="C90" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D90" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E90" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F90" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G90" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H90" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
logs: update NSE signals 2026-10-27
</commit_message>
<xml_diff>
--- a/logs/NSE_Bot_Master.xlsx
+++ b/logs/NSE_Bot_Master.xlsx
@@ -626,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X107"/>
+  <dimension ref="A1:X108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2854,9 +2854,16 @@
         </is>
       </c>
     </row>
+    <row r="108">
+      <c r="A108" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 2026-10-27  End of Day  |  Signals: 0  |  Stocks: None  ──</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V1"/>
-  <mergeCells count="87">
+  <mergeCells count="88">
     <mergeCell ref="A69:X69"/>
     <mergeCell ref="A78:X78"/>
     <mergeCell ref="A75:X75"/>
@@ -2880,6 +2887,7 @@
     <mergeCell ref="A82:X82"/>
     <mergeCell ref="A60:X60"/>
     <mergeCell ref="A25:X25"/>
+    <mergeCell ref="A108:X108"/>
     <mergeCell ref="A84:X84"/>
     <mergeCell ref="A66:X66"/>
     <mergeCell ref="A50:X50"/>
@@ -17030,7 +17038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I90"/>
+  <dimension ref="A1:I91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19762,6 +19770,36 @@
         <v>0</v>
       </c>
       <c r="H90" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="18" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B91" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="C91" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D91" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E91" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F91" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G91" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H91" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>